<commit_message>
Update Watchlists (Watchlists.xlsx) 2026-09-30 11:25
</commit_message>
<xml_diff>
--- a/data/Watchlists.xlsx
+++ b/data/Watchlists.xlsx
@@ -1,30 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://martincp1.sharepoint.com/sites/Eugene/Shared Documents/Operations/Scripts/Portfolio Dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8246B333-F41A-482E-89AE-B3C7B6FC1C48}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AE76102-C52C-42A9-844B-F6EA22AA1278}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="QDVD Watchlist A" sheetId="1" r:id="rId1"/>
-    <sheet name="QDVD Watchlist B" sheetId="2" r:id="rId2"/>
-    <sheet name="SMID Watchlist A" sheetId="3" r:id="rId3"/>
-    <sheet name="SMID Watchlist B" sheetId="4" r:id="rId4"/>
-    <sheet name="C Watch" sheetId="5" r:id="rId5"/>
+    <sheet name="PB_CACHE" sheetId="6" state="veryHidden" r:id="rId1"/>
+    <sheet name="QDVD Watchlist A" sheetId="1" r:id="rId2"/>
+    <sheet name="QDVD Watchlist B" sheetId="2" r:id="rId3"/>
+    <sheet name="SMID Watchlist A" sheetId="3" r:id="rId4"/>
+    <sheet name="SMID Watchlist B" sheetId="4" r:id="rId5"/>
+    <sheet name="C Watch" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="74">
   <si>
     <t>Ticker</t>
   </si>
@@ -240,6 +241,12 @@
   </si>
   <si>
     <t>WSO</t>
+  </si>
+  <si>
+    <t>PSX</t>
+  </si>
+  <si>
+    <t>H4sIAAAAAAAEAM2QTUvDQBCGt41iRH/E3g0hqf2wh1yMomAPlRQvpdTNMpilm924H0L6M/qHdTekevDg1RnYmVl4n3kZNEAIfbrw1cfl0D3PS2ZodSvlDq/aBjResFIR1Ub4BZRmUmSjZDSNU5dJhHPLjVWQCbBGER7hpS05o0/QruQORCYs56eeX3xjtx1222PjAhQjnO1JySEntILfP1cr2SzgA3g33TFqnA2nDRz3rHcV5rJuiAIVPhJdFWwPKEDhYVC02kAd55Jz6HQ6fgDhNtBjvX+3bptpj4DXdL3uVYVRTLxFuNZUKs7KnxuM48Tn3wcoZzMyoZNpOr8eQ3Iz32zCYX/u86BvTnzzH616cxdfI+bElycCAAA=</t>
   </si>
 </sst>
 </file>
@@ -611,6 +618,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA8F1C34-E096-44A3-8EB8-5BBA5EEF2316}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -642,7 +664,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -671,7 +693,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -700,7 +722,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -728,9 +750,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:A69"/>
+  <dimension ref="A1:A70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1081,18 +1103,28 @@
         <v>71</v>
       </c>
     </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1309,23 +1341,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F23C73-979C-443E-9CA2-7121B6C69145}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1350,12 +1380,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F23C73-979C-443E-9CA2-7121B6C69145}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
-    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Watchlists (Watchlists.xlsx) 2026-10-16 08:22
</commit_message>
<xml_diff>
--- a/data/Watchlists.xlsx
+++ b/data/Watchlists.xlsx
@@ -1,31 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://martincp1.sharepoint.com/sites/Eugene/Shared Documents/Operations/Scripts/Portfolio Dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AE76102-C52C-42A9-844B-F6EA22AA1278}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{784EC09C-D63D-40F4-9BE7-E18C71700A1D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="PB_CACHE" sheetId="6" state="veryHidden" r:id="rId1"/>
-    <sheet name="QDVD Watchlist A" sheetId="1" r:id="rId2"/>
-    <sheet name="QDVD Watchlist B" sheetId="2" r:id="rId3"/>
-    <sheet name="SMID Watchlist A" sheetId="3" r:id="rId4"/>
-    <sheet name="SMID Watchlist B" sheetId="4" r:id="rId5"/>
+    <sheet name="QDVD Watchlist A" sheetId="1" r:id="rId1"/>
+    <sheet name="QDVD Watchlist B" sheetId="2" r:id="rId2"/>
+    <sheet name="SMID Watchlist A" sheetId="3" r:id="rId3"/>
+    <sheet name="SMID Watchlist B" sheetId="4" r:id="rId4"/>
+    <sheet name="PB_CACHE" sheetId="7" state="veryHidden" r:id="rId5"/>
     <sheet name="C Watch" sheetId="5" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="75">
   <si>
     <t>Ticker</t>
   </si>
@@ -247,6 +260,9 @@
   </si>
   <si>
     <t>H4sIAAAAAAAEAM2QTUvDQBCGt41iRH/E3g0hqf2wh1yMomAPlRQvpdTNMpilm924H0L6M/qHdTekevDg1RnYmVl4n3kZNEAIfbrw1cfl0D3PS2ZodSvlDq/aBjResFIR1Ub4BZRmUmSjZDSNU5dJhHPLjVWQCbBGER7hpS05o0/QruQORCYs56eeX3xjtx1222PjAhQjnO1JySEntILfP1cr2SzgA3g33TFqnA2nDRz3rHcV5rJuiAIVPhJdFWwPKEDhYVC02kAd55Jz6HQ6fgDhNtBjvX+3bptpj4DXdL3uVYVRTLxFuNZUKs7KnxuM48Tn3wcoZzMyoZNpOr8eQ3Iz32zCYX/u86BvTnzzH616cxdfI+bElycCAAA=</t>
+  </si>
+  <si>
+    <t>J</t>
   </si>
 </sst>
 </file>
@@ -618,21 +634,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA8F1C34-E096-44A3-8EB8-5BBA5EEF2316}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -664,7 +665,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -693,7 +694,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -722,7 +723,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -750,9 +751,24 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8AE74AE-4548-4326-9CF7-372B551A4C6E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:A70"/>
+  <dimension ref="A1:A71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1106,6 +1122,11 @@
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
         <v>72</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" s="3" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1128,6 +1149,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
     <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
@@ -1340,15 +1370,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
   <ds:schemaRefs>
@@ -1361,6 +1382,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F23C73-979C-443E-9CA2-7121B6C69145}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A7D093A-965A-49F4-B796-FB43CAA20C7E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1377,12 +1406,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F23C73-979C-443E-9CA2-7121B6C69145}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Watchlists (Watchlists.xlsx) 2026-10-21 10:37
</commit_message>
<xml_diff>
--- a/data/Watchlists.xlsx
+++ b/data/Watchlists.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://martincp1.sharepoint.com/sites/Eugene/Shared Documents/Operations/Scripts/Portfolio Dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{784EC09C-D63D-40F4-9BE7-E18C71700A1D}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4156A0F-46DD-43E7-AC27-2AFEC0543B2E}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="QDVD Watchlist A" sheetId="1" r:id="rId1"/>
-    <sheet name="QDVD Watchlist B" sheetId="2" r:id="rId2"/>
-    <sheet name="SMID Watchlist A" sheetId="3" r:id="rId3"/>
-    <sheet name="SMID Watchlist B" sheetId="4" r:id="rId4"/>
-    <sheet name="PB_CACHE" sheetId="7" state="veryHidden" r:id="rId5"/>
+    <sheet name="PB_CACHE" sheetId="8" state="veryHidden" r:id="rId1"/>
+    <sheet name="QDVD Watchlist A" sheetId="1" r:id="rId2"/>
+    <sheet name="QDVD Watchlist B" sheetId="2" r:id="rId3"/>
+    <sheet name="SMID Watchlist A" sheetId="3" r:id="rId4"/>
+    <sheet name="SMID Watchlist B" sheetId="4" r:id="rId5"/>
     <sheet name="C Watch" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="77">
   <si>
     <t>Ticker</t>
   </si>
@@ -263,6 +263,12 @@
   </si>
   <si>
     <t>J</t>
+  </si>
+  <si>
+    <t>XYL</t>
+  </si>
+  <si>
+    <t>HTH</t>
   </si>
 </sst>
 </file>
@@ -633,7 +639,44 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="5">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{020EBD5E-9753-41CC-85A6-7CA7618FDB10}">
+  <we:reference id="29673e3c-d826-4f00-92ee-162334a52b1a" version="1.0.0.8" store="EXCatalog" storeType="EXCatalog"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;ca013001-a857-4e50-95ed-5b997cf1af42&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6687DEAB-51A6-4629-992D-51D95F2337CE}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -665,7 +708,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -694,7 +737,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -723,9 +766,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -746,23 +789,13 @@
         <v>40</v>
       </c>
     </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8AE74AE-4548-4326-9CF7-372B551A4C6E}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -961,172 +994,172 @@
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>59</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>4</v>
+        <v>60</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" s="2" t="s">
-        <v>63</v>
+      <c r="A62" s="3" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1135,6 +1168,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
@@ -1146,15 +1188,6 @@
     <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1371,20 +1404,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F23C73-979C-443E-9CA2-7121B6C69145}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
     <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F23C73-979C-443E-9CA2-7121B6C69145}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update Watchlists (Watchlists.xlsx) 2026-10-28 12:47
</commit_message>
<xml_diff>
--- a/data/Watchlists.xlsx
+++ b/data/Watchlists.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://martincp1.sharepoint.com/sites/Eugene/Shared Documents/Operations/Scripts/Portfolio Dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4156A0F-46DD-43E7-AC27-2AFEC0543B2E}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7F39B83-D4B4-4C88-A4A5-D85B3BD1ACDF}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PB_CACHE" sheetId="8" state="veryHidden" r:id="rId1"/>
@@ -723,7 +723,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -768,7 +768,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -781,7 +781,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -789,11 +789,6 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -801,7 +796,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:A71"/>
+  <dimension ref="A1:A72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1162,6 +1157,11 @@
         <v>76</v>
       </c>
     </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1177,20 +1177,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
     <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
@@ -1403,6 +1389,20 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F23C73-979C-443E-9CA2-7121B6C69145}">
   <ds:schemaRefs>
@@ -1412,17 +1412,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
-    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A7D093A-965A-49F4-B796-FB43CAA20C7E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1439,4 +1428,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>